<commit_message>
Added ways to save the models
</commit_message>
<xml_diff>
--- a/DropCore/OverallStatsDropCore-noboot.xlsx
+++ b/DropCore/OverallStatsDropCore-noboot.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alexb\OneDrive\Documents\Thesis\DropCore\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FD4522A-1594-4D9D-82A0-16ADBCAE40DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7907391-E4CD-4E9E-B64B-8213B2164635}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4060" yWindow="4060" windowWidth="28800" windowHeight="14460" xr2:uid="{84A3B88E-B226-40B3-A64E-0FDCC502A4B5}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{84A3B88E-B226-40B3-A64E-0FDCC502A4B5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="27">
   <si>
     <t>HalfCache</t>
   </si>
@@ -90,6 +90,33 @@
   </si>
   <si>
     <t>Facesim Drop 10</t>
+  </si>
+  <si>
+    <t>Nu: 0.5, Gamma: 0.99</t>
+  </si>
+  <si>
+    <t>Balanced Accuracy</t>
+  </si>
+  <si>
+    <t>Nu: 0.2, Gamma: 0.5</t>
+  </si>
+  <si>
+    <t>Facesim Drop 3</t>
+  </si>
+  <si>
+    <t>Streamcluster Drop 1</t>
+  </si>
+  <si>
+    <t>Nu: 0.1, Gamma: 0.5</t>
+  </si>
+  <si>
+    <t>Streamcluster Drop 10</t>
+  </si>
+  <si>
+    <t>Nu: 0.05, Gamma: 0.7</t>
+  </si>
+  <si>
+    <t>Streamcluster Drop 3</t>
   </si>
 </sst>
 </file>
@@ -461,7 +488,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{652EE7E4-9A64-4328-97BF-22E9AA604A6A}">
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:N34"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="34.36328125" customWidth="1"/>
@@ -470,12 +497,12 @@
     <col min="11" max="11" width="14.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -515,8 +542,11 @@
       <c r="M2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -560,8 +590,12 @@
       <c r="M5">
         <v>40</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N5">
+        <f>(K5+I5)/2</f>
+        <v>0.97788773523685912</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -605,80 +639,208 @@
       <c r="M6">
         <v>40</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="H7" t="e">
+      <c r="N6">
+        <f t="shared" ref="N6:N13" si="4">(K6+I6)/2</f>
+        <v>0.97788549418984205</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7">
+        <v>22</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>1335</v>
+      </c>
+      <c r="G7">
+        <v>99.926362297496297</v>
+      </c>
+      <c r="H7">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I7" t="e">
+        <v>1</v>
+      </c>
+      <c r="I7">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J7" t="e">
+        <v>0.95652173913043481</v>
+      </c>
+      <c r="J7">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K7" t="e">
+        <v>0.97777777777777775</v>
+      </c>
+      <c r="K7">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="H8" t="e">
+        <v>0.99925149700598803</v>
+      </c>
+      <c r="L7">
+        <v>0</v>
+      </c>
+      <c r="M7">
+        <v>40</v>
+      </c>
+      <c r="N7">
+        <f t="shared" si="4"/>
+        <v>0.97788661806821142</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8">
+        <v>10</v>
+      </c>
+      <c r="D8">
+        <v>2</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>954</v>
+      </c>
+      <c r="G8">
+        <v>99.7929606625258</v>
+      </c>
+      <c r="H8">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I8" t="e">
+        <v>1</v>
+      </c>
+      <c r="I8">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J8" t="e">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="J8">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K8" t="e">
+        <v>0.90909090909090906</v>
+      </c>
+      <c r="K8">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="H9" t="e">
+        <v>0.997907949790795</v>
+      </c>
+      <c r="L8">
+        <v>10</v>
+      </c>
+      <c r="M8">
+        <v>40</v>
+      </c>
+      <c r="N8">
+        <f t="shared" si="4"/>
+        <v>0.91562064156206424</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9">
+        <v>10</v>
+      </c>
+      <c r="D9">
+        <v>2</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <v>1389</v>
+      </c>
+      <c r="G9">
+        <v>99.786019969999998</v>
+      </c>
+      <c r="H9">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I9" t="e">
+        <v>0.90909090909090906</v>
+      </c>
+      <c r="I9">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J9" t="e">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="J9">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K9" t="e">
+        <v>0.86956521739130432</v>
+      </c>
+      <c r="K9">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="H10" t="e">
+        <v>0.99856218547807329</v>
+      </c>
+      <c r="L9">
+        <v>10</v>
+      </c>
+      <c r="M9">
+        <v>40</v>
+      </c>
+      <c r="N9">
+        <f t="shared" si="4"/>
+        <v>0.91594775940570328</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10">
+        <v>11</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>1135</v>
+      </c>
+      <c r="G10">
+        <v>99.912816041848302</v>
+      </c>
+      <c r="H10">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I10" t="e">
+        <v>1</v>
+      </c>
+      <c r="I10">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J10" t="e">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="J10">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K10" t="e">
+        <v>0.95652173913043481</v>
+      </c>
+      <c r="K10">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+        <v>0.99911971830985913</v>
+      </c>
+      <c r="L10">
+        <v>10</v>
+      </c>
+      <c r="M10">
+        <v>40</v>
+      </c>
+      <c r="N10">
+        <f t="shared" si="4"/>
+        <v>0.95789319248826288</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="H11" t="e">
         <f t="shared" si="1"/>
         <v>#DIV/0!</v>
@@ -695,8 +857,12 @@
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N11" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
       <c r="H12" t="e">
         <f t="shared" si="1"/>
         <v>#DIV/0!</v>
@@ -713,8 +879,12 @@
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N12" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
       <c r="H13" t="e">
         <f t="shared" si="1"/>
         <v>#DIV/0!</v>
@@ -730,6 +900,130 @@
       <c r="K13" t="e">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
+      </c>
+      <c r="N13" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>15</v>
+      </c>
+      <c r="B29">
+        <v>99.926578559999996</v>
+      </c>
+      <c r="C29">
+        <v>1</v>
+      </c>
+      <c r="D29">
+        <v>0.95652173913043481</v>
+      </c>
+      <c r="E29">
+        <v>0.97777777777777775</v>
+      </c>
+      <c r="F29">
+        <v>0.97788773523685912</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>17</v>
+      </c>
+      <c r="B30">
+        <v>99.92614476</v>
+      </c>
+      <c r="C30">
+        <v>1</v>
+      </c>
+      <c r="D30">
+        <v>0.95652173913043481</v>
+      </c>
+      <c r="E30">
+        <v>0.97777777777777775</v>
+      </c>
+      <c r="F30">
+        <v>0.97788549418984205</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>21</v>
+      </c>
+      <c r="B31">
+        <v>99.926362297496297</v>
+      </c>
+      <c r="C31">
+        <v>1</v>
+      </c>
+      <c r="D31">
+        <v>0.95652173913043481</v>
+      </c>
+      <c r="E31">
+        <v>0.97777777777777775</v>
+      </c>
+      <c r="F31">
+        <v>0.97788661806821142</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>22</v>
+      </c>
+      <c r="B32">
+        <v>99.7929606625258</v>
+      </c>
+      <c r="C32">
+        <v>1</v>
+      </c>
+      <c r="D32">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="E32">
+        <v>0.90909090909090906</v>
+      </c>
+      <c r="F32">
+        <v>0.91562064156206424</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>24</v>
+      </c>
+      <c r="B33">
+        <v>99.786019969999998</v>
+      </c>
+      <c r="C33">
+        <v>0.90909090909090906</v>
+      </c>
+      <c r="D33">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="E33">
+        <v>0.86956521739130432</v>
+      </c>
+      <c r="F33">
+        <v>0.91594775940570328</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>26</v>
+      </c>
+      <c r="B34">
+        <v>99.912816041848302</v>
+      </c>
+      <c r="C34">
+        <v>1</v>
+      </c>
+      <c r="D34">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="E34">
+        <v>0.95652173913043481</v>
+      </c>
+      <c r="F34">
+        <v>0.95789319248826288</v>
       </c>
     </row>
   </sheetData>

</xml_diff>